<commit_message>
running version with all dilution factors
</commit_message>
<xml_diff>
--- a/Einwagen.xlsx
+++ b/Einwagen.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Laufende_Projekte\Project_PGE\PGE_ID_conc_calc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\Laufende_Projekte\Project_PGE\PGE_ID\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95203AAF-B10F-40D8-8FBF-C08B69A04868}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851CC684-A862-4D3F-8FCA-A245C4B6B178}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11925" xr2:uid="{DFAE9E4B-DED2-4D02-9538-14C27B848607}"/>
   </bookViews>
@@ -26,25 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
-  <si>
-    <t>Spike 1</t>
-  </si>
-  <si>
-    <t>Spike 2</t>
-  </si>
-  <si>
-    <t>Calib_Spike_1-2</t>
-  </si>
-  <si>
-    <t>Calib_Spike_2-2</t>
-  </si>
-  <si>
-    <t>Calib_Spike_3-2</t>
-  </si>
-  <si>
-    <t>Calib_Spike_4-2</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>date</t>
   </si>
@@ -59,6 +41,33 @@
   </si>
   <si>
     <t>EW_gesamt</t>
+  </si>
+  <si>
+    <t>Calib_1</t>
+  </si>
+  <si>
+    <t>Calib_Spike_1</t>
+  </si>
+  <si>
+    <t>Calib_Spike_2</t>
+  </si>
+  <si>
+    <t>Calib_Spike_3</t>
+  </si>
+  <si>
+    <t>Calib_Spike_4</t>
+  </si>
+  <si>
+    <t>Calib_2</t>
+  </si>
+  <si>
+    <t>Calib_3</t>
+  </si>
+  <si>
+    <t>Spike_1</t>
+  </si>
+  <si>
+    <t>Spike_2</t>
   </si>
 </sst>
 </file>
@@ -428,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C9BD48-CD22-4E0E-8F4B-88C629425627}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" style="1" customWidth="1"/>
@@ -437,27 +446,27 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3">
-        <v>45194</v>
+        <v>45176</v>
       </c>
       <c r="D2" s="1">
         <v>1.0078</v>
@@ -470,10 +479,10 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3">
-        <v>45195</v>
+        <v>45176</v>
       </c>
       <c r="D3" s="1">
         <v>1.0105</v>
@@ -484,10 +493,10 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B4" s="3">
-        <v>45196</v>
+        <v>45176</v>
       </c>
       <c r="C4" s="1">
         <v>1.0039</v>
@@ -501,10 +510,10 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3">
-        <v>45197</v>
+        <v>45176</v>
       </c>
       <c r="C5" s="1">
         <v>1.0039</v>
@@ -518,10 +527,10 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B6" s="3">
-        <v>45198</v>
+        <v>45176</v>
       </c>
       <c r="C6" s="1">
         <v>1.0047999999999999</v>
@@ -535,10 +544,10 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B7" s="3">
-        <v>45199</v>
+        <v>45176</v>
       </c>
       <c r="C7" s="1">
         <v>1.0033000000000001</v>
@@ -548,6 +557,48 @@
       </c>
       <c r="E7" s="1">
         <v>10.0342</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="3">
+        <v>45176</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1.004</v>
+      </c>
+      <c r="E8" s="1">
+        <v>10.044700000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="3">
+        <v>45176</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1.0037</v>
+      </c>
+      <c r="E9" s="1">
+        <v>10.0381</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="3">
+        <v>45176</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1.0073000000000001</v>
+      </c>
+      <c r="E10" s="1">
+        <v>10.0328</v>
       </c>
     </row>
   </sheetData>

</xml_diff>